<commit_message>
docs(ucp): improve hours estimation
</commit_message>
<xml_diff>
--- a/docs/UseCasePoints_entrega2.xlsx
+++ b/docs/UseCasePoints_entrega2.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,8 +62,18 @@
       <color rgb="00FFFFFF"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="007F5000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="007F5000"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -88,6 +98,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002E75B6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -117,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -167,6 +182,11 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -532,7 +552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -686,11 +706,11 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Hours of Effort per Use Case Point</t>
+          <t>Hours per UCP — adjusted for academic part-time team and MVP scope</t>
         </is>
       </c>
       <c r="E15" s="6" t="n">
-        <v>4187</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16">
@@ -699,12 +719,47 @@
           <t>Hours of Effort</t>
         </is>
       </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Estimated Effort (hours)</t>
+        </is>
+      </c>
       <c r="E16" s="5" t="n">
-        <v>5516</v>
-      </c>
+        <v>1743</v>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>Nota</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>El ratio estándar de Schneider &amp; Winters (28 h/UCP) corresponde a equipos profesionales full-time. Para este proyecto se utiliza 8 h/UCP, ajustado al contexto académico (equipo de 5 estudiantes part-time, semestre de ~16 semanas) y al alcance de MVP del producto, alineándose con el rango referencial para MVPs Django comerciales (800–2.500 h).</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="n"/>
+      <c r="D18" s="19" t="n"/>
+      <c r="E18" s="19" t="n"/>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="19" t="n"/>
+      <c r="B19" s="19" t="n"/>
+      <c r="C19" s="19" t="n"/>
+      <c r="D19" s="19" t="n"/>
+      <c r="E19" s="19" t="n"/>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="19" t="n"/>
+      <c r="B20" s="19" t="n"/>
+      <c r="C20" s="19" t="n"/>
+      <c r="D20" s="19" t="n"/>
+      <c r="E20" s="19" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
+    <mergeCell ref="B18:E20"/>
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A1:E1"/>
@@ -721,7 +776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="B1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="2" max="2"/>
@@ -1053,7 +1108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="B1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="2" max="2"/>

</xml_diff>